<commit_message>
added processing for data testing ML
</commit_message>
<xml_diff>
--- a/ML_SSW_2025/Analysis_ML_Data.xlsx
+++ b/ML_SSW_2025/Analysis_ML_Data.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Desktop\ML_SSW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Desktop\InvestigacionUSFQ\SSWCompleteAnalysis\SingleSolitaryWaveAnalysis\ML_SSW_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C48F1D-EE23-448F-8878-C1E6DDD75E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA80105-062F-4B38-AE8E-CB5EEAED542C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AA4ED9E8-B08C-461E-9CA5-C3521FC84154}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{AA4ED9E8-B08C-461E-9CA5-C3521FC84154}"/>
   </bookViews>
   <sheets>
     <sheet name="Original Data" sheetId="1" r:id="rId1"/>
     <sheet name="ML_Example" sheetId="2" r:id="rId2"/>
     <sheet name="ML_TrainingData" sheetId="3" r:id="rId3"/>
+    <sheet name="ML_TestData_Ceramica" sheetId="4" r:id="rId4"/>
+    <sheet name="Ajuste_K" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="67">
   <si>
     <t>F1</t>
   </si>
@@ -146,6 +148,99 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>Probeta</t>
+  </si>
+  <si>
+    <t>Energía</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Golpes</t>
+  </si>
+  <si>
+    <t>M1 - Mod</t>
+  </si>
+  <si>
+    <t>M2 - Mod</t>
+  </si>
+  <si>
+    <t>M3 - Mod</t>
+  </si>
+  <si>
+    <t>M1 - Est</t>
+  </si>
+  <si>
+    <t>M2 - Est</t>
+  </si>
+  <si>
+    <t>M3 - Est</t>
+  </si>
+  <si>
+    <t>M4 - Est</t>
+  </si>
+  <si>
+    <t>M4 - Mod</t>
+  </si>
+  <si>
+    <t>M5 - Mod</t>
+  </si>
+  <si>
+    <t>M6 - Mod</t>
+  </si>
+  <si>
+    <t>M5 - Est</t>
+  </si>
+  <si>
+    <t>M6 - Est</t>
+  </si>
+  <si>
+    <t>TOF Prom</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>Den. Seca</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>g/cm3</t>
+  </si>
+  <si>
+    <t>25 golpes mod</t>
+  </si>
+  <si>
+    <t>MAX</t>
+  </si>
+  <si>
+    <t>DENSIDAD</t>
+  </si>
+  <si>
+    <t>56 golpes mod</t>
+  </si>
+  <si>
+    <t>25 golpes standard</t>
+  </si>
+  <si>
+    <t>Datos Matlab 0.1</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>Datos Matlab 0.3</t>
+  </si>
+  <si>
+    <t>Datos Matlab 0.5</t>
   </si>
 </sst>
 </file>
@@ -156,7 +251,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,8 +276,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="4"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -207,8 +327,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -240,13 +372,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -281,6 +426,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2985,4 +3140,973 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B6664A1-1E84-4EEF-A331-E575C33F569C}">
+  <dimension ref="A1:R21"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="16384" width="9.06640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.13911993692717059</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1.6982865896324033</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1.6584291622044007</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.11843409316154611</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="L2" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="1">
+        <v>3</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1.763728134637909</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0.11805225653206648</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" s="2">
+        <v>25</v>
+      </c>
+      <c r="M3" s="1">
+        <v>1.3520135201360978E-3</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0.11843409316154611</v>
+      </c>
+      <c r="O3" s="1">
+        <v>1.6584291622044007</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="R3" s="1">
+        <v>0.13911993692717059</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="1">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1.6822689096024417</v>
+      </c>
+      <c r="H4" s="1">
+        <v>9.6678107984795758E-2</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="2">
+        <v>56</v>
+      </c>
+      <c r="M4" s="1">
+        <v>1.3180131801320259E-3</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0.11805225653206648</v>
+      </c>
+      <c r="O4" s="1">
+        <v>1.763728134637909</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="R4" s="1">
+        <v>1.6982865896324033</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="1">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1.6483733962172045</v>
+      </c>
+      <c r="H5" s="1">
+        <v>8.0713111267325499E-2</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" s="2">
+        <v>56</v>
+      </c>
+      <c r="M5" s="1">
+        <v>1.2780127801285319E-3</v>
+      </c>
+      <c r="N5" s="1">
+        <v>9.6678107984795758E-2</v>
+      </c>
+      <c r="O5" s="1">
+        <v>1.6822689096024417</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1.62</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1.480677915463195</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0.11589041095890402</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L6" s="2">
+        <v>56</v>
+      </c>
+      <c r="M6" s="1">
+        <v>1.2380123801243302E-3</v>
+      </c>
+      <c r="N6" s="1">
+        <v>8.0713111267325499E-2</v>
+      </c>
+      <c r="O6" s="1">
+        <v>1.6483733962172045</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1.62</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1.4904689597154233</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0.13460442691211932</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L7" s="2">
+        <v>25</v>
+      </c>
+      <c r="M7" s="1">
+        <v>1.8960189601884298E-3</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0.11589041095890402</v>
+      </c>
+      <c r="O7" s="1">
+        <v>1.480677915463195</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1.62</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1.5294344523239138</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0.14028029887536533</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" s="2">
+        <v>25</v>
+      </c>
+      <c r="M8" s="1">
+        <v>1.83601836018994E-3</v>
+      </c>
+      <c r="N8" s="1">
+        <v>0.13460442691211932</v>
+      </c>
+      <c r="O8" s="1">
+        <v>1.4904689597154233</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="R8" s="1">
+        <v>0.13300000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1.62</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1.5475074537777984</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0.15156950672645753</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L9" s="2">
+        <v>25</v>
+      </c>
+      <c r="M9" s="1">
+        <v>1.4240142401433782E-3</v>
+      </c>
+      <c r="N9" s="1">
+        <v>0.14028029887536533</v>
+      </c>
+      <c r="O9" s="1">
+        <v>1.5294344523239138</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="R9" s="1">
+        <v>1.7749999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="1">
+        <v>3</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.7772421994397172</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0.1430861723446894</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L10" s="2">
+        <v>25</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1.6520165201640679E-3</v>
+      </c>
+      <c r="N10" s="1">
+        <v>0.15156950672645753</v>
+      </c>
+      <c r="O10" s="1">
+        <v>1.5475074537777984</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="1">
+        <v>3</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1.6951263354634258</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0.17279256442754556</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="1">
+        <v>3</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1.6321784584194605</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0.1863437537080784</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1.62</v>
+      </c>
+      <c r="G13" s="1">
+        <v>1.6090048691339709</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0.16556028504471754</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="L13" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="R13" s="1">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1.62</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1.6060302554528956</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0.19470446643487566</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L14" s="2">
+        <v>56</v>
+      </c>
+      <c r="M14" s="1">
+        <v>1.3240132401346459E-3</v>
+      </c>
+      <c r="N14" s="1">
+        <v>0.1430861723446894</v>
+      </c>
+      <c r="O14" s="1">
+        <v>1.7772421994397172</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="R14" s="1">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="1">
+        <v>2</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0.13911993692717059</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1.6982865896324033</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1.6867190368361413</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0.13297332509443671</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L15" s="2">
+        <v>56</v>
+      </c>
+      <c r="M15" s="1">
+        <v>1.484014840148264E-3</v>
+      </c>
+      <c r="N15" s="1">
+        <v>0.17279256442754556</v>
+      </c>
+      <c r="O15" s="1">
+        <v>1.6951263354634258</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="1">
+        <v>2</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.13911993692717059</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1.6982865896324033</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1.678484887889131</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0.15578764142732804</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="L16" s="2">
+        <v>56</v>
+      </c>
+      <c r="M16" s="1">
+        <v>1.5760157601505359E-3</v>
+      </c>
+      <c r="N16" s="1">
+        <v>0.1863437537080784</v>
+      </c>
+      <c r="O16" s="1">
+        <v>1.6321784584194605</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="1">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.13911993692717059</v>
+      </c>
+      <c r="F17" s="1">
+        <v>1.6982865896324033</v>
+      </c>
+      <c r="G17" s="1">
+        <v>1.601954608561813</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0.16935064935064942</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="L17" s="2">
+        <v>25</v>
+      </c>
+      <c r="M17" s="1">
+        <v>1.686016860168494E-3</v>
+      </c>
+      <c r="N17" s="1">
+        <v>0.16556028504471754</v>
+      </c>
+      <c r="O17" s="1">
+        <v>1.6090048691339709</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="K18" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L18" s="2">
+        <v>25</v>
+      </c>
+      <c r="M18" s="1">
+        <v>1.9700197001942142E-3</v>
+      </c>
+      <c r="N18" s="1">
+        <v>0.19470446643487566</v>
+      </c>
+      <c r="O18" s="1">
+        <v>1.6060302554528956</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="K19" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L19" s="2">
+        <v>25</v>
+      </c>
+      <c r="M19" s="1">
+        <v>1.4060140601390699E-3</v>
+      </c>
+      <c r="N19" s="1">
+        <v>0.13297332509443671</v>
+      </c>
+      <c r="O19" s="1">
+        <v>1.6867190368361413</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="K20" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L20" s="2">
+        <v>25</v>
+      </c>
+      <c r="M20" s="1">
+        <v>1.516015160152762E-3</v>
+      </c>
+      <c r="N20" s="1">
+        <v>0.15578764142732804</v>
+      </c>
+      <c r="O20" s="1">
+        <v>1.678484887889131</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="K21" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L21" s="2">
+        <v>25</v>
+      </c>
+      <c r="M21" s="1">
+        <v>1.455014550145075E-3</v>
+      </c>
+      <c r="N21" s="1">
+        <v>0.16935064935064942</v>
+      </c>
+      <c r="O21" s="1">
+        <v>1.601954608561813</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDBDB9C2-512F-468A-9E95-0283D0C33914}">
+  <dimension ref="B2:C33"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="2" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="B2" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="18"/>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="6">
+        <v>10000000</v>
+      </c>
+      <c r="C4" s="6">
+        <v>1.4007381733822328</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B5" s="6">
+        <v>40000000</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1.2140668286409155</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B6" s="6">
+        <v>100000000</v>
+      </c>
+      <c r="C6" s="6">
+        <v>1.1177048296059127</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B7" s="6">
+        <v>200000000</v>
+      </c>
+      <c r="C7" s="6">
+        <v>1.0909213561826436</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B8" s="6">
+        <v>300000000</v>
+      </c>
+      <c r="C8" s="6">
+        <v>1.08058437749855</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B9" s="6">
+        <v>500000000</v>
+      </c>
+      <c r="C9" s="6">
+        <v>1.0723113034395499</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B10" s="6">
+        <v>700000000</v>
+      </c>
+      <c r="C10" s="6">
+        <v>1.0694334868948585</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B11" s="6">
+        <v>1000000000</v>
+      </c>
+      <c r="C11" s="6">
+        <v>1.0629208338167233</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+    </row>
+    <row r="13" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="B13" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="18"/>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B15" s="6">
+        <v>10000000</v>
+      </c>
+      <c r="C15" s="6">
+        <v>1.3259736795022041</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B16" s="6">
+        <v>40000000</v>
+      </c>
+      <c r="C16" s="6">
+        <v>1.1531017802399695</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B17" s="6">
+        <v>100000000</v>
+      </c>
+      <c r="C17" s="6">
+        <v>1.0821813204036701</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B18" s="6">
+        <v>200000000</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1.05394888195359</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B19" s="6">
+        <v>300000000</v>
+      </c>
+      <c r="C19" s="6">
+        <v>1.0434829598242401</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B20" s="6">
+        <v>500000000</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1.0350255733857601</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B21" s="6">
+        <v>700000000</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1.0306193761935976</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B22" s="6">
+        <v>1000000000</v>
+      </c>
+      <c r="C22" s="6">
+        <v>1.0245285302824279</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+    </row>
+    <row r="24" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="B24" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="18"/>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B25" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B26" s="6">
+        <v>10000000</v>
+      </c>
+      <c r="C26" s="6">
+        <v>1.2535678601649396</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B27" s="6">
+        <v>40000000</v>
+      </c>
+      <c r="C27" s="6">
+        <v>1.0971579631994441</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B28" s="6">
+        <v>100000000</v>
+      </c>
+      <c r="C28" s="6">
+        <v>1.0400670315095699</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B29" s="6">
+        <v>200000000</v>
+      </c>
+      <c r="C29" s="6">
+        <v>1.0169791360217704</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B30" s="6">
+        <v>300000000</v>
+      </c>
+      <c r="C30" s="6">
+        <v>1.00942182278415</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B31" s="6">
+        <v>500000000</v>
+      </c>
+      <c r="C31" s="6">
+        <v>0.99776030496475798</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B32" s="6">
+        <v>700000000</v>
+      </c>
+      <c r="C32" s="6">
+        <v>0.98765618756805007</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B33" s="6">
+        <v>1000000000</v>
+      </c>
+      <c r="C33" s="6">
+        <v>0.97950536977613056</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B24:C24"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>